<commit_message>
Hygiene: blur coordinates in the HelioScope report, strip local path from the Excel download, move setup notes out of public, HSTS includeSubDomains and COOP; role targets tidy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/tools/advanced-excel/115-kWp-commercial-rooftop-excel-demo.xlsx
+++ b/public/tools/advanced-excel/115-kWp-commercial-rooftop-excel-demo.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usama\Desktop\Advanced Excel project\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{BFD6A18C-6BF6-47A7-A93D-FEB0AAD399EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12960" activeTab="3" xr2:uid="{CCF523AD-CD48-4FEF-8704-59CF0B6E4609}"/>

</xml_diff>